<commit_message>
Expand framing multiplex matrix with missing transport frames
</commit_message>
<xml_diff>
--- a/reports/framing_multiplex_matrix.xlsx
+++ b/reports/framing_multiplex_matrix.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -1381,6 +1381,2778 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>lifespan.startup</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ASGI lifespan receive frame</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>lifespan</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>event loop / worker instance</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>startup</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Process lifecycle, not request multiplexed</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>ASGI lifespan receive event required for FastAPI startup resources</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>lifespan.startup.complete</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ASGI lifespan send frame</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>lifespan</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>event loop / worker instance</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>startup complete</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Process lifecycle, not request multiplexed</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>ASGI lifespan success response</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>lifespan.startup.failed</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ASGI lifespan send frame</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>lifespan</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>event loop / worker instance</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>startup failed</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Process lifecycle, not request multiplexed</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Carries optional message and should stop startup</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>lifespan.shutdown</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ASGI lifespan receive frame</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>lifespan</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>event loop / worker instance</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>shutdown</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Process lifecycle, not request multiplexed</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>ASGI lifespan shutdown receive event</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>lifespan.shutdown.complete</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>ASGI lifespan send frame</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>lifespan</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>event loop / worker instance</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>shutdown complete</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Process lifecycle, not request multiplexed</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>ASGI lifespan shutdown success response</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>lifespan.shutdown.failed</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>ASGI lifespan send frame</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>lifespan</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>event loop / worker instance</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>shutdown failed</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Process lifecycle, not request multiplexed</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Carries optional message and should terminate with failure</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>http.request.body chunk</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>ASGI HTTP payload frame</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Partially represented</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>rest; jsonrpc; http.stream; sse</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>request scope</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>body + more_body</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Request body streaming</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Current event type exists but body/more_body payload schema is missing</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>http.response.start frame</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>ASGI HTTP response metadata frame</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Partially represented</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>rest; jsonrpc; http.stream; sse</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>request scope</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>status + headers + trailers flag</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Response metadata</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Current event type exists but status/headers/trailers payload schema is missing</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>http.response.body chunk</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>ASGI HTTP payload frame</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Partially represented</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>rest; jsonrpc; http.stream; sse</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>request scope</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>body + more_body</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Response body streaming</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Current event type exists but body/more_body payload schema is missing</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>http.response.trailers</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>ASGI HTTP trailer frame</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>rest; jsonrpc; http.stream; sse</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>request scope</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>headers + more_trailers</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Trailer metadata after body</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Required when http.response.start trailers=true</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>websocket.accept frame</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>ASGI WebSocket handshake frame</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Partially represented</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>websocket</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>connection scope</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>subprotocol + headers</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Handshake state transition</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Current event type exists but payload schema is missing</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>websocket.receive.text</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>ASGI WebSocket data frame</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Partially represented</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>websocket</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>connection scope</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Duplex message stream</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Requires text/bytes exclusivity schema</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>websocket.receive.bytes</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>ASGI WebSocket data frame</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Partially represented</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>websocket</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>connection scope</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>bytes</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Duplex message stream</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Requires text/bytes exclusivity schema</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>websocket.send.text</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>ASGI WebSocket data frame</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Partially represented</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>websocket</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>connection scope</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Duplex message stream</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Requires text/bytes exclusivity schema</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>websocket.send.bytes</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>ASGI WebSocket data frame</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Partially represented</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>websocket</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>connection scope</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>bytes</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Duplex message stream</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Requires text/bytes exclusivity schema</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>websocket.close frame</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>ASGI WebSocket close frame</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Partially represented</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>websocket</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>connection scope</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>code + reason</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Connection close</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Current event type exists but code/reason payload schema is missing</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>websocket.disconnect frame</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>ASGI WebSocket disconnect frame</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Partially represented</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>websocket</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>connection scope</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>code + reason</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Connection close observation</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Current event type exists but code/reason payload schema is missing</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>WebSocket ping frame</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>WebSocket control frame</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Not exposed by ASGI app</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>websocket</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>connection scope</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>opcode ping</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Protocol keepalive</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Usually handled by server; track as server-managed frame</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>WebSocket pong frame</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>WebSocket control frame</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Not exposed by ASGI app</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>websocket</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>connection scope</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>opcode pong</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Protocol keepalive</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Usually handled by server; track as server-managed frame</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>WebSocket continuation frame</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>WebSocket fragmentation frame</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Not exposed by ASGI app</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>websocket</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>connection scope</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>opcode continuation</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Fragment assembly</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Server should deliver complete messages to ASGI app</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>ASGI TLS extension</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>scope extension metadata</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Partially represented</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>http; websocket</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>connection scope</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>extensions.tls</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>No multiplexing</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Current ext.transport.tls is not aligned to ASGI TLS extension fields</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>mTLS client certificate chain</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>TLS extension metadata</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>http; websocket</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>connection scope</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>client_cert_chain</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>No multiplexing</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Needed for client certificate identity and verification evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>proxy forwarded headers</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>deployment metadata frame</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>http; websocket</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>trusted proxy hop chain</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Forwarded / X-Forwarded-* / X-Real-IP</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Proxy chain derivation</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Needed to distinguish raw vs effective scheme/client/server/root_path</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>PROXY protocol v1 line</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>load balancer transport preface</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>http; websocket</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>connection preface</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>PROXY TCP4/TCP6/UNKNOWN</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Connection metadata before HTTP</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Not an HTTP header; should be separate from forwarded headers</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>PROXY protocol v2 binary header</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>load balancer transport preface</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>http; websocket</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>connection preface</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>signature + command + TLVs</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Connection metadata before HTTP</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Binary proxy metadata including SSL TLVs</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>HTTP/2 DATA frame</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>HTTP/2 protocol frame</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Not explicit</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>http bindings over h2</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>stream_id</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>DATA</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Native HTTP stream multiplex</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Maps to ASGI body chunks after server normalization</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>HTTP/2 HEADERS frame</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>HTTP/2 protocol frame</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Not explicit</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>http bindings over h2</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>stream_id</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>HEADERS</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Native HTTP stream multiplex</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Maps to ASGI scope headers or response start/trailers</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>HTTP/2 RST_STREAM frame</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>HTTP/2 control frame</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>http bindings over h2</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>stream_id</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>RST_STREAM error code</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Stream cancellation</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Needed for abort/cancel semantics</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>HTTP/2 SETTINGS frame</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>HTTP/2 control frame</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>http bindings over h2</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>connection</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>SETTINGS identifiers</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Connection-level control</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Server/client capability and flow-control metadata</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>HTTP/2 PUSH_PROMISE frame</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>HTTP/2 server push frame</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>http bindings over h2</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>promised stream_id</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>PUSH_PROMISE</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Server push multiplex</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Not modeled in current contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>HTTP/2 PING frame</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>HTTP/2 control frame</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>http bindings over h2</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>connection</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>PING opaque data</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Connection keepalive</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Protocol-level health frame</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>HTTP/2 GOAWAY frame</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>HTTP/2 control frame</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>http bindings over h2</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>last_stream_id</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>GOAWAY error code</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Connection drain</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Needed for graceful connection shutdown semantics</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>HTTP/2 WINDOW_UPDATE frame</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>HTTP/2 flow-control frame</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>http bindings over h2</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>connection or stream_id</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>window increment</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Flow-control multiplex</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Needed for backpressure/flow-control profile</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>HTTP/2 CONTINUATION frame</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>HTTP/2 header block frame</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>http bindings over h2</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>stream_id</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>CONTINUATION</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Header block continuation</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Server should normalize before ASGI headers</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>HTTP/3 DATA frame</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>HTTP/3 protocol frame</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Not explicit</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>http bindings over h3</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>QUIC stream identity</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>DATA</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Native HTTP stream multiplex over QUIC</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Maps to ASGI body chunks after server normalization</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>HTTP/3 HEADERS frame</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>HTTP/3 protocol frame</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Not explicit</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>http bindings over h3</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>QUIC stream identity</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>HEADERS</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Native HTTP stream multiplex over QUIC</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Maps to ASGI scope headers or response start/trailers</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>HTTP/3 SETTINGS frame</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>HTTP/3 control frame</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>http bindings over h3</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>control stream</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>SETTINGS identifiers</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Connection-level control</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>H3 capability metadata</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>HTTP/3 PUSH_PROMISE frame</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>HTTP/3 server push frame</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>http bindings over h3</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>push id</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>PUSH_PROMISE</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Server push multiplex</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Not modeled in current contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>HTTP/3 CANCEL_PUSH frame</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>HTTP/3 control frame</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>http bindings over h3</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>push id</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>CANCEL_PUSH</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Server push cancellation</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Not modeled in current contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>HTTP/3 GOAWAY frame</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>HTTP/3 control frame</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>http bindings over h3</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>stream id / push id</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>GOAWAY</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Connection drain</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Needed for graceful connection shutdown semantics</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>HTTP/3 MAX_PUSH_ID frame</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>HTTP/3 control frame</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>http bindings over h3</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>push id</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>MAX_PUSH_ID</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Server push control</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Not modeled in current contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>HTTP/3 DATAGRAM frame</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>HTTP/3 extension frame</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>http bindings over h3; webtransport</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>quarter stream id / context id</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>H3 DATAGRAM</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Unreliable datagram multiplex</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Distinct from WebTransport datagram application event</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>QUIC RESET_STREAM frame</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>QUIC transport frame</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>webtransport; h3</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>stream_id</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>application error code + final size</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Transport stream cancellation</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Needed for WebTransport stream reset semantics</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>QUIC STOP_SENDING frame</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>QUIC transport frame</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>webtransport; h3</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>stream_id</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>application error code</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Transport stream cancellation</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Peer stop-sending signal</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>QUIC CONNECTION_CLOSE frame</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>QUIC transport frame</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>webtransport; h3</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>connection</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>error code + reason</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Connection close</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Needed for QUIC close reason semantics</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>QUIC PATH_CHALLENGE frame</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>QUIC transport frame</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>webtransport; h3</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>path</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>challenge data</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Path validation</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Needed for migration/path validation profile</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>QUIC PATH_RESPONSE frame</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>QUIC transport frame</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>webtransport; h3</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>path</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>response data</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Path validation</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Needed for migration/path validation profile</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>QUIC NEW_CONNECTION_ID frame</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>QUIC transport frame</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>webtransport; h3</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>connection id sequence</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>connection id</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Connection migration support</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Needed for QUIC connection-id lifecycle</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>QUIC RETIRE_CONNECTION_ID frame</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>QUIC transport frame</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>webtransport; h3</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>connection id sequence</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>retire sequence</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Connection migration support</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Needed for QUIC connection-id lifecycle</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>SSE data field</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>SSE field frame</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Partially represented</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>sse</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>event stream</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Server event stream</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Currently collapsed into http.response.body</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>SSE event field</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>SSE field frame</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Partially represented</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>sse</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>event stream</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>event</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Server event discrimination</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Currently only ext.sse metadata exists</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>SSE id field</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>SSE field frame</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Partially represented</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>sse</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>event stream</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Replay/cursor key</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Currently only ext.sse.last_event_id exists</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>SSE retry field</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>SSE field frame</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Partially represented</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>sse</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>event stream</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>retry</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Reconnect policy</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Currently only ext.sse.retry_ms exists</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>SSE comment/heartbeat field</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>SSE field frame</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>sse</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>event stream</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>comment line</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Keepalive</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Needed to distinguish heartbeat comments from data events</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>JSON-RPC request object</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>JSON-RPC envelope frame</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Partially represented</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>jsonrpc; websocket; webtransport</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>method</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Request correlation multiplexing</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Current jsonrpc framing label has no envelope schema</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>JSON-RPC response object</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>JSON-RPC envelope frame</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Partially represented</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>jsonrpc; websocket; webtransport</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>result</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Request correlation multiplexing</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Current jsonrpc framing label has no envelope schema</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>JSON-RPC error object</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>JSON-RPC envelope frame</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Partially represented</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>jsonrpc; websocket; webtransport</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>error.code</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Request correlation multiplexing</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>Current jsonrpc framing label has no envelope schema</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>JSON-RPC notification object</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>JSON-RPC envelope frame</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Partially represented</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>jsonrpc; websocket; webtransport</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>method</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>no id</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Method dispatch without response</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Current jsonrpc framing label has no envelope schema</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>JSON-RPC batch array</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>JSON-RPC envelope frame</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>jsonrpc; websocket; webtransport</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>per item id/method</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>array envelope</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Batch multiplex inside one payload</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Needed for complete JSON-RPC coverage</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>multipart boundary frame</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>HTTP body subframing</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>rest; http.stream</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>boundary</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>part boundary</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Body part multiplex</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Needed for multipart/form-data and multipart/mixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>multipart part headers</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>HTTP body subframing</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>rest; http.stream</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>part index/name</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>part headers</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Body part metadata</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Needed for form/file upload schemas</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>multipart part body chunk</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>HTTP body subframing</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>rest; http.stream</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>part index/name</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>part body bytes</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Body part streaming</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Needed for file upload streaming</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>SVCB DNS record</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>service discovery record</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>service name</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>SvcPriority + TargetName + SvcParams</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Discovery metadata</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Advertises endpoint parameters such as alpn, port, ipv4hint, ipv6hint, ech</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>HTTPS DNS record</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>service discovery record</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>origin name</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>SvcPriority + TargetName + SvcParams</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Discovery metadata</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>HTTPS RR specialization of SVCB</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Alt-Svc header field</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>HTTP service advertisement</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>rest; jsonrpc; http.stream; sse</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>origin + alternative authority</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>alpn-id + authority + parameters</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>Alternative service discovery</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Advertises h2/h3 alternatives and max-age/persist parameters</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>ECHConfig SVCB parameter</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>service discovery parameter</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>service name</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>ech</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Discovery metadata</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Needed for Encrypted ClientHello advertisement tracking</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1392,7 +4164,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33" customWidth="1" min="1" max="1"/>
@@ -1642,6 +4414,1788 @@
       <c r="E9" s="2" t="inlineStr">
         <is>
           <t>tigrbl</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>lifespan.startup</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>event loop / worker instance</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>startup</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>lifespan</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>lifespan.startup.complete</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>event loop / worker instance</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>startup complete</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>lifespan</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>lifespan.startup.failed</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>event loop / worker instance</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>startup failed</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>lifespan</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>lifespan.shutdown</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>event loop / worker instance</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>shutdown</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>lifespan</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>lifespan.shutdown.complete</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>event loop / worker instance</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>shutdown complete</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>lifespan</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>lifespan.shutdown.failed</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>event loop / worker instance</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>shutdown failed</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>lifespan</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>http.request.body chunk</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>schema-hardening</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>request scope</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>body + more_body</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>rest; jsonrpc; http.stream; sse</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>http.response.start frame</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>schema-hardening</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>request scope</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>status + headers + trailers flag</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>rest; jsonrpc; http.stream; sse</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>http.response.body chunk</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>schema-hardening</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>request scope</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>body + more_body</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>rest; jsonrpc; http.stream; sse</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>http.response.trailers</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>request scope</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>headers + more_trailers</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>rest; jsonrpc; http.stream; sse</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>websocket.accept frame</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>schema-hardening</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>connection scope</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>subprotocol + headers</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>websocket</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>websocket.receive.text</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>schema-hardening</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>connection scope</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>websocket</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>websocket.receive.bytes</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>schema-hardening</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>connection scope</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>bytes</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>websocket</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>websocket.send.text</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>schema-hardening</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>connection scope</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>websocket</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>websocket.send.bytes</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>schema-hardening</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>connection scope</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>bytes</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>websocket</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>websocket.close frame</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>schema-hardening</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>connection scope</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>code + reason</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>websocket</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>websocket.disconnect frame</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>schema-hardening</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>connection scope</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>code + reason</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>websocket</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>WebSocket ping frame</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>schema-hardening</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>connection scope</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>opcode ping</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>websocket</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>WebSocket pong frame</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>schema-hardening</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>connection scope</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>opcode pong</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>websocket</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>WebSocket continuation frame</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>schema-hardening</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>connection scope</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>opcode continuation</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>websocket</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>ASGI TLS extension</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>schema-hardening</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>connection scope</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>extensions.tls</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>http; websocket</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>mTLS client certificate chain</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>connection scope</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>client_cert_chain</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>http; websocket</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>proxy forwarded headers</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>trusted proxy hop chain</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Forwarded / X-Forwarded-* / X-Real-IP</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>http; websocket</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>PROXY protocol v1 line</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>connection preface</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>PROXY TCP4/TCP6/UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>http; websocket</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>PROXY protocol v2 binary header</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>connection preface</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>signature + command + TLVs</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>http; websocket</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>HTTP/2 DATA frame</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>stream_id</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>DATA</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>http bindings over h2</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>HTTP/2 HEADERS frame</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>stream_id</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>HEADERS</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>http bindings over h2</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>HTTP/2 RST_STREAM frame</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>stream_id</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>RST_STREAM error code</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>http bindings over h2</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>HTTP/2 SETTINGS frame</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>connection</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>SETTINGS identifiers</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>http bindings over h2</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>HTTP/2 PUSH_PROMISE frame</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>promised stream_id</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>PUSH_PROMISE</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>http bindings over h2</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>HTTP/2 PING frame</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>connection</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>PING opaque data</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>http bindings over h2</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>HTTP/2 GOAWAY frame</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>last_stream_id</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>GOAWAY error code</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>http bindings over h2</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>HTTP/2 WINDOW_UPDATE frame</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>connection or stream_id</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>window increment</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>http bindings over h2</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>HTTP/2 CONTINUATION frame</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>stream_id</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>CONTINUATION</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>http bindings over h2</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>HTTP/3 DATA frame</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>QUIC stream identity</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>DATA</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>http bindings over h3</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>HTTP/3 HEADERS frame</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>QUIC stream identity</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>HEADERS</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>http bindings over h3</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>HTTP/3 SETTINGS frame</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>control stream</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>SETTINGS identifiers</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>http bindings over h3</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>HTTP/3 PUSH_PROMISE frame</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>push id</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>PUSH_PROMISE</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>http bindings over h3</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>HTTP/3 CANCEL_PUSH frame</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>push id</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>CANCEL_PUSH</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>http bindings over h3</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>HTTP/3 GOAWAY frame</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>stream id / push id</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>GOAWAY</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>http bindings over h3</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>HTTP/3 MAX_PUSH_ID frame</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>push id</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>MAX_PUSH_ID</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>http bindings over h3</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>HTTP/3 DATAGRAM frame</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>quarter stream id / context id</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>H3 DATAGRAM</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>http bindings over h3; webtransport</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>QUIC RESET_STREAM frame</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>stream_id</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>application error code + final size</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>webtransport; h3</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>QUIC STOP_SENDING frame</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>stream_id</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>application error code</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>webtransport; h3</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>QUIC CONNECTION_CLOSE frame</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>connection</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>error code + reason</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>webtransport; h3</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>QUIC PATH_CHALLENGE frame</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>path</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>challenge data</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>webtransport; h3</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>QUIC PATH_RESPONSE frame</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>path</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>response data</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>webtransport; h3</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>QUIC NEW_CONNECTION_ID frame</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>connection id sequence</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>connection id</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>webtransport; h3</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>QUIC RETIRE_CONNECTION_ID frame</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>connection id sequence</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>retire sequence</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>webtransport; h3</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>SSE data field</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>schema-hardening</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>event stream</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>sse</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>SSE event field</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>schema-hardening</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>event stream</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>event</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>sse</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>SSE id field</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>schema-hardening</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>event stream</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>sse</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>SSE retry field</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>schema-hardening</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>event stream</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>retry</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>sse</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>SSE comment/heartbeat field</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>event stream</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>comment line</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>sse</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>JSON-RPC request object</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>schema-hardening</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>method</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>jsonrpc; websocket; webtransport</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>JSON-RPC response object</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>schema-hardening</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>result</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>jsonrpc; websocket; webtransport</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>JSON-RPC error object</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>schema-hardening</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>error.code</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>jsonrpc; websocket; webtransport</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>JSON-RPC notification object</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>schema-hardening</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>method</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>no id</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>jsonrpc; websocket; webtransport</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>JSON-RPC batch array</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>per item id/method</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>array envelope</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>jsonrpc; websocket; webtransport</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>multipart boundary frame</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>boundary</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>part boundary</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>rest; http.stream</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>multipart part headers</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>part index/name</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>part headers</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>rest; http.stream</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>multipart part body chunk</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>part index/name</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>part body bytes</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>rest; http.stream</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>SVCB DNS record</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>service name</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>SvcPriority + TargetName + SvcParams</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>HTTPS DNS record</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>origin name</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>SvcPriority + TargetName + SvcParams</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Alt-Svc header field</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>origin + alternative authority</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>alpn-id + authority + parameters</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>rest; jsonrpc; http.stream; sse</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>ECHConfig SVCB parameter</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>service name</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>ech</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>none</t>
         </is>
       </c>
     </row>

</xml_diff>